<commit_message>
Some tweaks to B and D revs.
</commit_message>
<xml_diff>
--- a/Mussel_heartrate_daughterboard/Mussel_heartrate_daughterboard_parts.xlsx
+++ b/Mussel_heartrate_daughterboard/Mussel_heartrate_daughterboard_parts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Hardware_projects\MusselHeartRate\Mussel_heartrate_daughterboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382A44B1-1EE0-4623-AECD-5007437DA0BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA6848B-743D-448D-AD13-E566D8E10D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2870" yWindow="1400" windowWidth="30060" windowHeight="14480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36240" yWindow="830" windowWidth="27130" windowHeight="19680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RevAB_parts" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="HeartRate_Daughterboard_RevA_bom" localSheetId="1">RevA_BOM!$A$2:$G$48</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -31,7 +31,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -93,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="206">
   <si>
     <t>Digikey.com materials</t>
   </si>
@@ -705,6 +704,12 @@
   </si>
   <si>
     <t>SSM3J328RLFCT-ND</t>
+  </si>
+  <si>
+    <t>WM9021-ND</t>
+  </si>
+  <si>
+    <t>Molex KK PremiumGrade Hand Crimp Tool for Mini-Fit Jr. 22-28AWG</t>
   </si>
 </sst>
 </file>
@@ -1158,7 +1163,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1169,7 +1174,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.90625" customWidth="1"/>
@@ -2154,6 +2159,23 @@
       <c r="J37" s="19">
         <f>SUM(J31:J35)</f>
         <v>557.15319999999997</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>205</v>
+      </c>
+      <c r="B40">
+        <v>638190800</v>
+      </c>
+      <c r="C40" t="s">
+        <v>204</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40" s="20">
+        <v>401.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>